<commit_message>
Criado as classes Account e BookStore Pages
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -116,8 +116,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="3">
     <font>
+      <sz val="12.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -130,15 +137,21 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor theme="0" tint="-0.499984740745262"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -146,19 +159,35 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -728,83 +757,86 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Criado metodos autorização e gerarToken na classe AccountPage
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -91,40 +91,57 @@
     <t>UserTest</t>
   </si>
   <si>
+    <t>Tester</t>
+  </si>
+  <si>
+    <t>tgo.user@mail.com</t>
+  </si>
+  <si>
+    <t>123@Abcd</t>
+  </si>
+  <si>
+    <t>9781491904244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You Don't Know JS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kyle Simpson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O'Reilly Media</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>UserDev</t>
+  </si>
+  <si>
     <t>Dev</t>
   </si>
   <si>
     <t>tgo.dev@mail.com</t>
   </si>
   <si>
-    <t>123@Abcd</t>
-  </si>
-  <si>
-    <t>9781491904244</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You Don't Know JS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kyle Simpson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O'Reilly Media</t>
+    <t>9781449325862</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Git Pocket Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richard E. Silverman</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="12.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -137,21 +154,15 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.499984740745262"/>
-        <bgColor theme="0" tint="-0.499984740745262"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -159,36 +170,19 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -746,97 +740,129 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="3" max="3" width="27.625"/>
-    <col bestFit="1" min="4" max="4" width="11.25390625"/>
-    <col bestFit="1" min="6" max="6" width="16.0625"/>
-    <col bestFit="1" min="7" max="7" width="10.125"/>
-    <col customWidth="1" min="9" max="9" width="32.625"/>
-    <col bestFit="1" min="10" max="10" width="24.5625"/>
-    <col bestFit="1" min="11" max="11" width="11.43359375"/>
+    <col bestFit="1" min="6" max="6" width="16.68359375"/>
+    <col customWidth="1" min="9" max="9" width="17.75390625"/>
+    <col bestFit="1" min="10" max="10" width="15.75390625"/>
+    <col bestFit="1" min="11" max="11" width="17.125"/>
     <col bestFit="1" min="12" max="12" width="12.18359375"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="N2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Refatorado todos os metodos na classe AccountPage
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -162,12 +162,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
       <diagonal style="none"/>
     </border>
   </borders>
@@ -176,12 +191,10 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -748,89 +761,91 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="H2" s="1"/>
+      <c r="I2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N2" t="s">
+      <c r="M2" s="1"/>
+      <c r="N2" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="4">
@@ -839,7 +854,7 @@
       <c r="C3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -851,18 +866,21 @@
       <c r="G3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="H3" s="1"/>
+      <c r="I3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Concluido criação do cenario 01
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -79,7 +79,7 @@
     <t>PUBLISHER</t>
   </si>
   <si>
-    <t>TOTALPAGES</t>
+    <t>PAGES</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
@@ -128,9 +128,6 @@
     <t xml:space="preserve">O'Reilly Media</t>
   </si>
   <si>
-    <t>278</t>
-  </si>
-  <si>
     <t xml:space="preserve">No matter how much experience you have with JavaScript, odds are you don’t fully understand the language. As part of the \"You Don’t Know JS\" series, this compact guide focuses on new features available in ECMAScript 6 (ES6), the latest version of the st</t>
   </si>
   <si>
@@ -165,13 +162,28 @@
     <t xml:space="preserve">Richard E. Silverman</t>
   </si>
   <si>
-    <t>`234</t>
-  </si>
-  <si>
     <t xml:space="preserve">This pocket guide is the perfect on-the-job companion to Git, the distributed version control system. It provides a compact, readable introduction to Git for new users, as well as a reference to common commands and procedures for those of you with Git exp</t>
   </si>
   <si>
     <t>http://chimera.labs.oreilly.com/books/1230000000561/index.html</t>
+  </si>
+  <si>
+    <t>9781449331818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learning JavaScript Design Patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A JavaScript and jQuery Developer's Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addy Osmani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With Learning JavaScript Design Patterns, you'll learn how to write beautiful, structured, and maintainable JavaScript by applying classical and modern design patterns to the language. If you want to keep your code efficient, more manageable, and up-to-da</t>
+  </si>
+  <si>
+    <t>http://www.addyosmani.com/resources/essentialjsdesignpatterns/book/</t>
   </si>
 </sst>
 </file>
@@ -227,11 +239,8 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -241,8 +250,9 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -846,7 +856,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
@@ -855,13 +865,13 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
@@ -887,20 +897,20 @@
       <c r="E2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>23</v>
       </c>
       <c r="H2" s="1"/>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="L2" s="1" t="s">
@@ -909,74 +919,126 @@
       <c r="M2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="3">
+        <v>278</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="Q2" s="1"/>
       <c r="R2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" ht="66">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="5">
+        <v>2</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="6">
-        <v>2</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="1"/>
+      <c r="I3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="3">
+        <v>234</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>43</v>
       </c>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
+    </row>
+    <row r="4" ht="66">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="1">
+        <v>254</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2"/>
     <hyperlink r:id="rId2" ref="P3"/>
+    <hyperlink r:id="rId1" ref="F4"/>
+    <hyperlink r:id="rId3" ref="P4"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Corrigido erro no metodo removerTodosOsLivros()
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -95,7 +95,7 @@
     <t>ERRO</t>
   </si>
   <si>
-    <t>Sim</t>
+    <t>Não</t>
   </si>
   <si>
     <t xml:space="preserve">Validar adicionar livro ao perfil</t>
@@ -139,9 +139,6 @@
     <t/>
   </si>
   <si>
-    <t>Não</t>
-  </si>
-  <si>
     <t>UserDev</t>
   </si>
   <si>
@@ -209,6 +206,9 @@
   </si>
   <si>
     <t>NEW_WEBSITE</t>
+  </si>
+  <si>
+    <t>Sim</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmar que livro foi atualizado</t>
@@ -306,9 +306,12 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -963,153 +966,153 @@
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="3"/>
+      <c r="I2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="5">
         <v>278</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2" t="s">
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" ht="66">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="5">
-        <v>2</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="5">
+        <v>234</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" s="4">
-        <v>234</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="P3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4" ht="66">
-      <c r="A4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="4" t="s">
+      <c r="H4" s="3"/>
+      <c r="I4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="3">
+        <v>254</v>
+      </c>
+      <c r="O4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="2">
-        <v>254</v>
-      </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1192,28 +1195,28 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>16</v>
@@ -1224,153 +1227,153 @@
     </row>
     <row r="2" ht="132">
       <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="2">
+        <v>55</v>
+      </c>
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2">
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
         <v>9781491904244</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="3">
         <v>278</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" s="3">
+        <v>254</v>
+      </c>
+      <c r="W2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="V2" s="2">
-        <v>254</v>
-      </c>
-      <c r="W2" s="2" t="s">
+      <c r="X2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="X2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Y2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="2"/>
+      <c r="Z2" s="3"/>
     </row>
     <row r="3" ht="99">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="5">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="3">
+        <v>234</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" s="2">
-        <v>234</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="R3" s="9" t="s">
+      <c r="R3" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="S3" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="T3" s="9" t="s">
+      <c r="T3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="U3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="V3" s="9">
+      <c r="V3" s="10">
         <v>352</v>
       </c>
-      <c r="W3" s="9" t="s">
+      <c r="W3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X3" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Corrigido erro que gerava token nulo
</commit_message>
<xml_diff>
--- a/test-data/cenarios_e_massas.xlsx
+++ b/test-data/cenarios_e_massas.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Cenário 1" sheetId="1" state="visible" r:id="rId2"/>
@@ -95,7 +95,7 @@
     <t>ERRO</t>
   </si>
   <si>
-    <t>Não</t>
+    <t>Sim</t>
   </si>
   <si>
     <t xml:space="preserve">Validar adicionar livro ao perfil</t>
@@ -139,6 +139,9 @@
     <t/>
   </si>
   <si>
+    <t>Não</t>
+  </si>
+  <si>
     <t>UserDev</t>
   </si>
   <si>
@@ -206,9 +209,6 @@
   </si>
   <si>
     <t>NEW_WEBSITE</t>
-  </si>
-  <si>
-    <t>Sim</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmar que livro foi atualizado</t>
@@ -314,14 +314,15 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -966,57 +967,57 @@
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="5" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="4">
         <v>278</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3" t="s">
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" ht="66">
-      <c r="A3" s="6" t="s">
-        <v>18</v>
+      <c r="A3" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
@@ -1025,94 +1026,94 @@
         <v>19</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" s="3" t="s">
+      <c r="H3" s="2"/>
+      <c r="I3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="L3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="4">
         <v>234</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>39</v>
+      <c r="O3" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+        <v>41</v>
+      </c>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
     </row>
     <row r="4" ht="66">
-      <c r="A4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="3">
+      <c r="A4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="3" t="s">
+      <c r="H4" s="2"/>
+      <c r="I4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="K4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="L4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="3">
+      <c r="N4" s="2">
         <v>254</v>
       </c>
-      <c r="O4" s="3" t="s">
-        <v>45</v>
+      <c r="O4" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+        <v>47</v>
+      </c>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1195,28 +1196,28 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>16</v>
@@ -1226,127 +1227,127 @@
       </c>
     </row>
     <row r="2" ht="132">
-      <c r="A2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="3">
+      <c r="A2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2">
         <v>9781491904244</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="3">
+      <c r="N2" s="2">
         <v>278</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="R2" s="3" t="s">
+      <c r="Q2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="S2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="T2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="V2" s="3">
+      <c r="V2" s="2">
         <v>254</v>
       </c>
-      <c r="W2" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="X2" s="3" t="s">
+      <c r="W2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="X2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="3"/>
+      <c r="Z2" s="2"/>
     </row>
     <row r="3" ht="99">
-      <c r="A3" s="6" t="s">
-        <v>18</v>
+      <c r="A3" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>56</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" s="3" t="s">
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="L3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="2">
         <v>234</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" s="4" t="s">
+      <c r="O3" s="2" t="s">
         <v>40</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="Q3" s="9" t="s">
         <v>57</v>
@@ -1369,11 +1370,11 @@
       <c r="W3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="X3" s="3" t="s">
+      <c r="X3" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="3"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>